<commit_message>
zhihao is now former
</commit_message>
<xml_diff>
--- a/data/source_people.xlsx
+++ b/data/source_people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa77\Documents\.MIJN BESTANDEN\Wiskunde &amp; Informatica\NAS website\GitHub repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD146A73-98E7-490B-910A-EE29DE0D7B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97808E78-9633-4EC1-9202-4AE88021C12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="236">
   <si>
     <t>Prof.dr.ir.</t>
   </si>
@@ -480,12 +480,6 @@
     <t>E. Paramonova</t>
   </si>
   <si>
-    <t>former postDoc / professor</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
     <t>Annalisa Socievole</t>
   </si>
   <si>
@@ -718,6 +712,30 @@
   </si>
   <si>
     <t>B.L. Chang</t>
+  </si>
+  <si>
+    <t>name_abbrev2</t>
+  </si>
+  <si>
+    <t>N. Baken</t>
+  </si>
+  <si>
+    <t>Nico Baken</t>
+  </si>
+  <si>
+    <t>N.H.B. Baken</t>
+  </si>
+  <si>
+    <t>Former NAS Professor</t>
+  </si>
+  <si>
+    <t>R. Kooij</t>
+  </si>
+  <si>
+    <t>G. Balogh</t>
+  </si>
+  <si>
+    <t>B. Chang</t>
   </si>
 </sst>
 </file>
@@ -1076,17 +1094,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="24.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.77734375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="38.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="73.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.109375" style="4"/>
-    <col min="9" max="16384" width="9.109375" style="2"/>
+    <col min="3" max="4" width="22.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="38.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="73.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.109375" style="4"/>
+    <col min="10" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -1100,22 +1118,22 @@
         <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>151</v>
+      <c r="I1" s="6" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1123,22 +1141,22 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>206</v>
+      <c r="I2" s="4" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1151,22 +1169,22 @@
       <c r="C3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="4" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1178,22 +1196,22 @@
       <c r="C4" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3"/>
+      <c r="E4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1205,22 +1223,22 @@
       <c r="C5" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3"/>
+      <c r="E5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="4" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1232,22 +1250,22 @@
       <c r="C6" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3"/>
+      <c r="E6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="I6" s="4"/>
+      <c r="I6" s="4" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -1259,22 +1277,22 @@
       <c r="C7" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3"/>
+      <c r="E7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="I7" s="4"/>
+      <c r="I7" s="4" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -1286,44 +1304,46 @@
       <c r="C8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="I8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>184</v>
+        <v>166</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>212</v>
+        <v>182</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1331,22 +1351,23 @@
         <v>3</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="4" t="s">
         <v>169</v>
       </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="H10" s="4" t="s">
-        <v>220</v>
+        <v>167</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1359,41 +1380,41 @@
       <c r="C11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>202</v>
-      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="I11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D12" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>186</v>
+      <c r="G12" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>204</v>
+        <v>184</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1401,22 +1422,23 @@
         <v>21</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D13" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>205</v>
+      <c r="I13" s="4" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -1426,20 +1448,21 @@
       <c r="C14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3"/>
+      <c r="E14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>207</v>
+      <c r="I14" s="4" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -1449,60 +1472,61 @@
       <c r="C15" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3"/>
+      <c r="E15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>209</v>
+      <c r="I15" s="4" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D16" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>185</v>
+      <c r="G16" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>211</v>
+        <v>183</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D17" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>187</v>
+      <c r="G17" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>214</v>
+        <v>185</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -1512,60 +1536,62 @@
       <c r="C18" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3"/>
+      <c r="E18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>215</v>
+      <c r="I18" s="4" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B19" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D19" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>189</v>
+      <c r="G19" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>219</v>
+        <v>187</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D20" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>190</v>
+      <c r="G20" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>221</v>
+        <v>188</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
@@ -1575,20 +1601,21 @@
       <c r="C21" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3"/>
+      <c r="E21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>222</v>
+      <c r="I21" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -1598,20 +1625,21 @@
       <c r="C22" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3"/>
+      <c r="E22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>223</v>
+      <c r="I22" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -1621,20 +1649,21 @@
       <c r="C23" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="3"/>
+      <c r="E23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>225</v>
+      <c r="I23" s="4" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -1644,40 +1673,41 @@
       <c r="C24" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3"/>
+      <c r="E24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="H24" s="4" t="s">
-        <v>226</v>
+      <c r="I24" s="4" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D25" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>188</v>
+      <c r="G25" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>227</v>
+        <v>186</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -1687,20 +1717,21 @@
       <c r="C26" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="D26" s="3"/>
       <c r="E26" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H26" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="H26" s="4" t="s">
-        <v>228</v>
+      <c r="I26" s="4" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -1711,12 +1742,12 @@
         <v>147</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1725,19 +1756,17 @@
         <v>3</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>150</v>
+        <v>157</v>
+      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -1750,14 +1779,11 @@
       <c r="C29" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>150</v>
+      <c r="E29" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -1765,19 +1791,16 @@
         <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -1785,19 +1808,16 @@
         <v>3</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -1805,62 +1825,53 @@
         <v>3</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>155</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E34" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>3</v>
       </c>
@@ -1868,19 +1879,16 @@
         <v>12</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>3</v>
       </c>
@@ -1890,20 +1898,18 @@
       <c r="C36" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>201</v>
-      </c>
+      <c r="D36" s="3"/>
       <c r="E36" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G36" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>3</v>
       </c>
@@ -1913,17 +1919,18 @@
       <c r="C37" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>199</v>
-      </c>
+      <c r="D37" s="3"/>
       <c r="E37" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F37" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G37" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>3</v>
       </c>
@@ -1933,17 +1940,18 @@
       <c r="C38" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>199</v>
-      </c>
+      <c r="D38" s="3"/>
       <c r="E38" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>3</v>
       </c>
@@ -1953,17 +1961,17 @@
       <c r="C39" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="E39" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F39" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G39" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>3</v>
       </c>
@@ -1973,17 +1981,18 @@
       <c r="C40" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>199</v>
-      </c>
+      <c r="D40" s="5"/>
       <c r="E40" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="G40" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>3</v>
       </c>
@@ -1993,14 +2002,14 @@
       <c r="C41" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>3</v>
       </c>
@@ -2010,17 +2019,17 @@
       <c r="C42" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="E42" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G42" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>3</v>
       </c>
@@ -2030,14 +2039,14 @@
       <c r="C43" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E43" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>3</v>
       </c>
@@ -2047,17 +2056,17 @@
       <c r="C44" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="E44" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G44" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>3</v>
       </c>
@@ -2067,14 +2076,14 @@
       <c r="C45" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E45" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>3</v>
       </c>
@@ -2084,17 +2093,18 @@
       <c r="C46" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>199</v>
-      </c>
+      <c r="D46" s="5"/>
       <c r="E46" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F46" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G46" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>3</v>
       </c>
@@ -2104,14 +2114,14 @@
       <c r="C47" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E47" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>3</v>
       </c>
@@ -2121,14 +2131,14 @@
       <c r="C48" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E48" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>3</v>
       </c>
@@ -2138,14 +2148,14 @@
       <c r="C49" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E49" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>3</v>
       </c>
@@ -2153,16 +2163,16 @@
         <v>100</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>3</v>
       </c>
@@ -2172,14 +2182,14 @@
       <c r="C51" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E51" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>3</v>
       </c>
@@ -2189,14 +2199,15 @@
       <c r="C52" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D52" s="5"/>
+      <c r="E52" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>3</v>
       </c>
@@ -2206,14 +2217,14 @@
       <c r="C53" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E53" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>3</v>
       </c>
@@ -2223,14 +2234,14 @@
       <c r="C54" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E54" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>3</v>
       </c>
@@ -2240,14 +2251,14 @@
       <c r="C55" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E55" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>3</v>
       </c>
@@ -2257,14 +2268,14 @@
       <c r="C56" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E56" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>3</v>
       </c>
@@ -2274,14 +2285,14 @@
       <c r="C57" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E57" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>3</v>
       </c>
@@ -2291,14 +2302,15 @@
       <c r="C58" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D58" s="5"/>
+      <c r="E58" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>3</v>
       </c>
@@ -2308,14 +2320,14 @@
       <c r="C59" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D59" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E59" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>3</v>
       </c>
@@ -2323,16 +2335,16 @@
         <v>119</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>3</v>
       </c>
@@ -2340,16 +2352,16 @@
         <v>120</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>3</v>
       </c>
@@ -2359,14 +2371,14 @@
       <c r="C62" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D62" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E62" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>3</v>
       </c>
@@ -2376,14 +2388,15 @@
       <c r="C63" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D63" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D63" s="5"/>
+      <c r="E63" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>3</v>
       </c>
@@ -2391,16 +2404,16 @@
         <v>125</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>3</v>
       </c>
@@ -2410,14 +2423,14 @@
       <c r="C65" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E65" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>3</v>
       </c>
@@ -2427,14 +2440,14 @@
       <c r="C66" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E66" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>3</v>
       </c>
@@ -2444,14 +2457,14 @@
       <c r="C67" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E67" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>3</v>
       </c>
@@ -2461,14 +2474,14 @@
       <c r="C68" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E68" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>3</v>
       </c>
@@ -2478,14 +2491,15 @@
       <c r="C69" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D69" s="5"/>
+      <c r="E69" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>3</v>
       </c>
@@ -2495,14 +2509,14 @@
       <c r="C70" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E70" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>3</v>
       </c>
@@ -2512,14 +2526,14 @@
       <c r="C71" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E71" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>3</v>
       </c>
@@ -2527,16 +2541,16 @@
         <v>140</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>3</v>
       </c>
@@ -2546,14 +2560,14 @@
       <c r="C73" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D73" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E73" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>3</v>
       </c>
@@ -2563,14 +2577,14 @@
       <c r="C74" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D74" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E74" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>3</v>
       </c>
@@ -2580,21 +2594,39 @@
       <c r="C75" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D75" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F75" s="2" t="s">
+      <c r="D75" s="5"/>
+      <c r="E75" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B76" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G76" s="2" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I75" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I75">
-      <sortCondition descending="1" ref="D1:D75"/>
+      <sortCondition descending="1" ref="E1:E75"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F20">
-    <sortCondition descending="1" ref="E3:E20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G20">
+    <sortCondition descending="1" ref="F3:F20"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
tick off some tasks
</commit_message>
<xml_diff>
--- a/data/source_people.xlsx
+++ b/data/source_people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa77\Documents\.MIJN BESTANDEN\Wiskunde &amp; Informatica\NAS website\GitHub repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15BC976-CD90-42D7-919A-4702CA398AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F120F0-FC63-4498-A74A-56F5214F133F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="234">
   <si>
     <t>Prof.dr.ir.</t>
   </si>
@@ -2597,6 +2597,9 @@
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="B76" s="2" t="s">
         <v>230</v>
       </c>

</xml_diff>

<commit_message>
cleanup various papers with spelling errors
</commit_message>
<xml_diff>
--- a/data/source_people.xlsx
+++ b/data/source_people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa77\Documents\.MIJN BESTANDEN\Wiskunde &amp; Informatica\NAS website\GitHub repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7D351C-6E12-48D0-AAC8-569E5581E125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C1B5ED-3D30-40B7-B078-42AD2BC907B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="237">
   <si>
     <t>Prof.dr.ir.</t>
   </si>
@@ -730,6 +730,15 @@
   </si>
   <si>
     <t>https://www.nas.ewi.tudelft.nl/images/profile_photos/Roberto%20Gheda.jpg</t>
+  </si>
+  <si>
+    <t>A. Beshir</t>
+  </si>
+  <si>
+    <t>J.M. Meier</t>
+  </si>
+  <si>
+    <t>J. Omić</t>
   </si>
 </sst>
 </file>
@@ -1995,6 +2004,9 @@
       <c r="C44" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="D44" s="2" t="s">
+        <v>235</v>
+      </c>
       <c r="E44" s="2" t="s">
         <v>197</v>
       </c>
@@ -2028,6 +2040,9 @@
       </c>
       <c r="C46" s="2" t="s">
         <v>131</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>197</v>
@@ -2577,6 +2592,9 @@
       </c>
       <c r="C74" s="2" t="s">
         <v>192</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>234</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>197</v>

</xml_diff>